<commit_message>
feat: add Project HTML Dashboard Export Engine v1
</commit_message>
<xml_diff>
--- a/outputs/projects/bruynzeel_waterfront/09_exports/bruynzeel_waterfront_project_tables.xlsx
+++ b/outputs/projects/bruynzeel_waterfront/09_exports/bruynzeel_waterfront_project_tables.xlsx
@@ -156,7 +156,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-24T17:41:12</t>
+          <t>2026-06-24T18:08:13</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-24T17:41:12</t>
+          <t>2026-06-24T18:08:13</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">

</xml_diff>

<commit_message>
feat: add Project Index Startpage Engine v1
</commit_message>
<xml_diff>
--- a/outputs/projects/bruynzeel_waterfront/09_exports/bruynzeel_waterfront_project_tables.xlsx
+++ b/outputs/projects/bruynzeel_waterfront/09_exports/bruynzeel_waterfront_project_tables.xlsx
@@ -156,7 +156,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-24T18:08:13</t>
+          <t>2026-06-24T18:47:18</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-24T18:08:13</t>
+          <t>2026-06-24T18:47:18</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">

</xml_diff>

<commit_message>
feat: add Project Audit Trail Engine v1
</commit_message>
<xml_diff>
--- a/outputs/projects/bruynzeel_waterfront/09_exports/bruynzeel_waterfront_project_tables.xlsx
+++ b/outputs/projects/bruynzeel_waterfront/09_exports/bruynzeel_waterfront_project_tables.xlsx
@@ -156,7 +156,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-24T18:47:18</t>
+          <t>2026-06-24T23:26:12</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-24T18:47:18</t>
+          <t>2026-06-24T23:26:12</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">

</xml_diff>

<commit_message>
feat: add Project Git Evidence Engine v1
</commit_message>
<xml_diff>
--- a/outputs/projects/bruynzeel_waterfront/09_exports/bruynzeel_waterfront_project_tables.xlsx
+++ b/outputs/projects/bruynzeel_waterfront/09_exports/bruynzeel_waterfront_project_tables.xlsx
@@ -156,7 +156,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-24T23:26:12</t>
+          <t>2026-06-25T00:16:12</t>
         </is>
       </c>
     </row>
@@ -396,12 +396,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -428,12 +428,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -460,12 +460,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -492,12 +492,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -524,12 +524,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -556,12 +556,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -588,12 +588,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -652,12 +652,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -684,12 +684,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -716,12 +716,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -748,12 +748,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -780,12 +780,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -812,12 +812,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -844,12 +844,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-11-26</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -876,12 +876,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-11-28</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-12-02</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-24T23:26:12</t>
+          <t>2026-06-25T00:16:12</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">

</xml_diff>

<commit_message>
feat: add auto repair engine and refresh project outputs
</commit_message>
<xml_diff>
--- a/outputs/projects/bruynzeel_waterfront/09_exports/bruynzeel_waterfront_project_tables.xlsx
+++ b/outputs/projects/bruynzeel_waterfront/09_exports/bruynzeel_waterfront_project_tables.xlsx
@@ -156,7 +156,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-25T00:16:12</t>
+          <t>2026-07-02T23:06:20</t>
         </is>
       </c>
     </row>
@@ -396,12 +396,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -428,12 +428,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -460,12 +460,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -492,12 +492,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -524,12 +524,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -556,12 +556,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -588,12 +588,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -652,12 +652,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -684,12 +684,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -716,12 +716,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -748,12 +748,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -780,12 +780,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -812,12 +812,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -844,12 +844,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -876,12 +876,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2026-12-05</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-12-02</t>
+          <t>2026-12-09</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-25T00:16:12</t>
+          <t>2026-07-02T23:06:20</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">

</xml_diff>

<commit_message>
feat: connect Building Technical Engine to BAOEES Core
</commit_message>
<xml_diff>
--- a/outputs/projects/bruynzeel_waterfront/09_exports/bruynzeel_waterfront_project_tables.xlsx
+++ b/outputs/projects/bruynzeel_waterfront/09_exports/bruynzeel_waterfront_project_tables.xlsx
@@ -156,7 +156,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-02T23:06:20</t>
+          <t>2026-07-03T11:31:34</t>
         </is>
       </c>
     </row>
@@ -396,12 +396,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -428,12 +428,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -460,12 +460,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -492,12 +492,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -524,12 +524,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -556,12 +556,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -588,12 +588,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -652,12 +652,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -684,12 +684,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -716,12 +716,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -748,12 +748,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -780,12 +780,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -812,12 +812,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -844,12 +844,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-12-04</t>
+          <t>2026-12-05</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -876,12 +876,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-12-05</t>
+          <t>2026-12-06</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-12-09</t>
+          <t>2026-12-10</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-02T23:06:20</t>
+          <t>2026-07-03T11:31:34</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">

</xml_diff>